<commit_message>
fix(schema): render CO's list as a bag with elements, as CO 2.0 does
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/uco.xlsx
+++ b/project/excel/uco.xlsx
@@ -837,13 +837,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>co_size</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>element</t>
         </is>
       </c>
     </row>
@@ -16814,7 +16819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16831,6 +16836,16 @@
       <c r="C1" t="inlineStr">
         <is>
           <t>lastItem</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>co_size</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>element</t>
         </is>
       </c>
     </row>
@@ -29718,7 +29733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29748,6 +29763,11 @@
         </is>
       </c>
       <c r="F1" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
         <is>
           <t>type</t>
         </is>

</xml_diff>